<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-01 Le camion rouge sur le tapis
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-01.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le garage au bout des coussins</t>
+          <t>Le camion rouge sur le tapis</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine puis salon, tartine et tapis</t>
+          <t>maison, salon, camion rouge, tapis bleu, parquet, rayon, sac, boîte en bois</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut que le camion rouge arrive au garage en bois. Victorina parle peu. Sarah lui tend le camion. Elles font une route de coussins. Le camion entre au garage.</t>
+          <t>Un rayon glisse sur le parquet. Près du tapis bleu, un éclat de parquet brille. Sarah veut le camion rouge, maintenant. Victorina ne dit rien. Sarah pousse trop vite. Sourire parti, poitrine, papa accroupi. Elle refuse de foncer, attend, tend le camion. Merci vécu. Boîte en bois, camion trop vite. Un éclat de parquet tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le couvercle du pot de confiture résiste. Un peu de fraise a collé au bord. Des miettes dorées sont sur la table. La tartine sent encore le pain chaud. Tu as vu la colle de fraise, Sarah ? Elle est rouge, papa. On tourne tout doux. Le couvercle part. Ça fait un petit toc. Sarah lèche un doigt. C'est sucré. Un peu, pas trop. Le camion rouge attend près du tapis. Ses roues sont un peu poussiéreuses. Le garage en bois est au bout du salon. La porte du garage est ouverte. En ce moment, Sarah pose un coussin. Puis un autre coussin. Je fais une route. Jusqu'au garage. Pour le camion rouge ? Oui. Il doit arriver. La porte s'ouvre. Victorina arrive avec son sac. Le sac frotte le parquet. Victorina parle peu. Elle regarde le sol. Sarah a envie de tout raconter. La tartine. La fraise. La route. Les mots montent très vite. On peut attendre. Tu peux tendre un jouet. Sarah tient le camion rouge. Les roues sont encore froides. Victorina ne dit rien.</t>
+          <t>Un rayon glisse sur le parquet. Ça fait une ligne chaude, étroite. Il chauffe le bois, papa. Tu le vois, le rayon, Sarah ? Oui, papa. Le tapis bleu tient un carré de soleil. Le poil est tiède, contre la paume. Il est chaud, maman. Le soleil est dessus ? Oui. Près du tapis, un éclat de parquet brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse dans le rayon. Elle vole, papa. Au-dessus du tapis ? Oui, au-dessus. Le camion rouge reste au bord du tapis. Ses roues sont froides, un peu poussiéreuses. Il sent le plastique, papa. Tu le tiens, Sarah ? Oui. En ce moment, Sarah pose le camion. Je veux le camion, maintenant ! Sur le tapis bleu, tout de suite. Une petite route, là ? Oui, une route. Les roues touchent le poil bleu. Il doit partir. La porte s'ouvre. Victorina arrive avec son sac. Le sac frotte le parquet. Elle regarde le sol. Elle ne dit rien. Tu pousses avec moi ? Victorina serre le sac. Sarah a envie de tout raconter. Les mots montent très vite. Le rayon ! Le tapis ! Le camion ! Sarah pousse trop vite vers elle. Le camion tape le sac. Oh. Le camion bascule sur le parquet. Le camion. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorina, Sarah ? Oui, papa. Tes mains tiennent le camion, Sarah ? Un peu, maman. L'éclat de parquet tremble, puis tient. Victorina reste près du sac. Elle ne dit rien, papa. Sarah regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le couvercle du pot de confiture résiste. Un peu de fraise a collé au bord. Des miettes dorées sont sur la table. La tartine sent encore le pain chaud. Tu as vu la colle de fraise, Sarah ? Elle est rouge, papa. On tourne tout doux. Le couvercle part. Ça fait un petit toc. Sarah lèche un doigt. C'est sucré. Un peu, pas trop. Le camion rouge attend près du tapis. Ses roues sont un peu poussiéreuses. Le garage en bois est au bout du salon. La porte du garage est ouverte. En ce moment, Sarah pose un coussin. Puis un autre coussin. Je fais une route. Jusqu'au garage. Pour le camion rouge ? Oui. Il doit arriver. La porte s'ouvre. Victorina arrive avec son sac. Le sac frotte le parquet. Victorina parle peu. Elle regarde le sol. Sarah a envie de tout raconter. La tartine. La fraise. La route. Les mots montent très vite. On peut attendre. Tu peux tendre un jouet. Sarah tient le camion rouge. Les roues sont encore froides. Victorina ne dit rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon glisse sur le parquet. Ça fait une ligne chaude, étroite. Il chauffe le bois, papa. Tu le vois, le rayon, Sarah ? Oui, papa. Le tapis bleu tient un carré de soleil. Le poil est tiède, contre la paume. Il est chaud, maman. Le soleil est dessus ? Oui. Près du tapis, un &lt;emphasis level="moderate"&gt;éclat de parquet&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse dans le rayon. Elle vole, papa. Au-dessus du tapis ? Oui, au-dessus. Le camion rouge reste au bord du tapis. Ses roues sont froides, un peu poussiéreuses. Il sent le plastique, papa. Tu le tiens, Sarah ? Oui. En ce moment, Sarah pose le camion. Je veux le camion, maintenant ! Sur le tapis bleu, tout de suite. Une petite route, là ? Oui, une route. Les roues touchent le poil bleu. Il doit partir. La porte s'ouvre. Victorina arrive avec son sac. Le sac frotte le parquet. Elle regarde le sol. Elle ne dit rien. Tu pousses avec moi ? Victorina serre le sac. Sarah a envie de tout raconter. Les mots montent très vite. Le rayon ! Le tapis ! Le camion ! Sarah pousse trop vite vers elle. Le camion tape le sac. Oh. Le camion bascule sur le parquet. Le camion. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorina, Sarah ? Oui, papa. Tes mains tiennent le camion, Sarah ? Un peu, maman. L'éclat de parquet tremble, puis tient. Victorina reste près du sac. Elle ne dit rien, papa. Sarah regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kenzo est dans le salon. Le tapis est doux. Maman ouvre la porte. Maya arrive avec son sac. Maya parle peu. Elle regarde le sol. Kenzo veut poser beaucoup de questions. Il ouvre la bouche. Maman dit doucement : on peut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. On n'imite pas. On ne va pas forcer la parole. Kenzo ferme la bouche. Il respire. Il prend un camion rouge. Il va tendre un jouet. Il tend le camion vers Maya. Maya regarde. Elle ne dit rien. Kenzo attend. Le salon est calme. On entend l'horloge. Maya prend le camion. Elle le fait rouler. Kenzo sourit. Il prend une petite voiture bleue. Il la pose près du camion. Maya pousse le camion. La voiture avance aussi. Ils font une route avec des coussins. Maya ne parle toujours pas. C'est possible. Maman dit : on peut attendre. On peut tendre un jouet. On ne va pas forcer la parole. Kenzo hoche la tête. Il tend un garage en bois. Maya le pose au bout de la route. Un silence. Puis Maya dit tout bas : vroom. Kenzo dit : vroom. Ils jouent. Plus tard, maman propose un goûter. Maya secoue la tête. Kenzo dit : d'accord. Maman dit : d'accord. Regarder, c'est bien aussi. Kenzo boit son verre. Maya reste près du tapis. Elle tient encore le camion. Kenzo attend. Puis Maya vient s'asseoir. Elle croque un morceau de pomme. Elle ne raconte rien. Kenzo range une voiture. Le jeu a eu lieu, même avec peu de mots. [pause]</t>
+          <t>Un rayon glisse sur le parquet. Ça fait une ligne chaude, étroite. Il chauffe le bois, papa. Tu le vois, le rayon, Sarah ? Oui, papa. Le tapis bleu tient un carré de soleil. Le poil est tiède, contre la paume. Il est chaud, maman. Le soleil est dessus ? Oui. Près du tapis, un &lt;emphasis&gt;éclat de parquet&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse dans le rayon. Elle vole, papa. Au-dessus du tapis ? Oui, au-dessus. Le camion rouge reste au bord du tapis. Ses roues sont froides, un peu poussiéreuses. Il sent le plastique, papa. Tu le tiens, Sarah ? Oui. En ce moment, Sarah pose le camion. Je veux le camion, maintenant ! Sur le tapis bleu, tout de suite. Une petite route, là ? Oui, une route. Les roues touchent le poil bleu. Il doit partir. La porte s'ouvre. Victorina arrive avec son sac. Le sac frotte le parquet. Elle regarde le sol. Elle ne dit rien. Tu pousses avec moi ? Victorina serre le sac. Sarah a envie de tout raconter. Les mots montent très vite. Le rayon ! Le tapis ! Le camion ! Sarah pousse trop vite vers elle. Le camion tape le sac. Oh. Le camion bascule sur le parquet. Le camion. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorina, Sarah ? Oui, papa. Tes mains tiennent le camion, Sarah ? Un peu, maman. L'éclat de parquet tremble, puis tient. Victorina reste près du sac. Elle ne dit rien, papa. Sarah regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de parquet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,47 +1326,77 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_camion_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le couvercle du pot de confiture résiste.
-narrateur|Un peu de fraise a collé au bord.
-narrateur|Des miettes dorées sont sur la table.
-narrateur|La tartine sent encore le pain chaud.
-papa|Tu as vu la colle de fraise, Sarah ?
-enfant-f|Elle est rouge, papa.
-maman|On tourne tout doux.
-narrateur|Le couvercle part.
-narrateur|Ça fait un petit toc.
-narrateur|Sarah lèche un doigt.
-enfant-f|C'est sucré.
-maman|Un peu, pas trop.
-narrateur|Le camion rouge attend près du tapis.
-narrateur|Ses roues sont un peu poussiéreuses.
-narrateur|Le garage en bois est au bout du salon.
-narrateur|La porte du garage est ouverte.
-narrateur|En ce moment, Sarah pose un coussin.
-narrateur|Puis un autre coussin.
-enfant-f|Je fais une route.
-enfant-f|Jusqu'au garage.
-papa|Pour le camion rouge ?
+          <t>narrateur|Un rayon glisse sur le parquet.
+narrateur|Ça fait une ligne chaude, étroite.
+enfant-f|Il chauffe le bois, papa.
+papa|Tu le vois, le rayon, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le tapis bleu tient un carré de soleil.
+narrateur|Le poil est tiède, contre la paume.
+enfant-f|Il est chaud, maman.
+maman|Le soleil est dessus ?
 enfant-f|Oui.
-enfant-f|Il doit arriver.
+narrateur|Près du tapis, un éclat de parquet brille.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Une poussière danse dans le rayon.
+enfant-f|Elle vole, papa.
+papa|Au-dessus du tapis ?
+enfant-f|Oui, au-dessus.
+narrateur|Le camion rouge reste au bord du tapis.
+narrateur|Ses roues sont froides, un peu poussiéreuses.
+enfant-f|Il sent le plastique, papa.
+papa|Tu le tiens, Sarah ?
+enfant-f|Oui.
+narrateur|En ce moment, Sarah pose le camion.
+enfant-f|Je veux le camion, maintenant !
+enfant-f|Sur le tapis bleu, tout de suite.
+papa|Une petite route, là ?
+enfant-f|Oui, une route.
+maman|Les roues touchent le poil bleu.
+enfant-f|Il doit partir.
 narrateur|La porte s'ouvre.
 narrateur|Victorina arrive avec son sac.
 narrateur|Le sac frotte le parquet.
-narrateur|Victorina parle peu.
 narrateur|Elle regarde le sol.
+narrateur|Elle ne dit rien.
+enfant-f|Tu pousses avec moi ?
+narrateur|Victorina serre le sac.
 narrateur|Sarah a envie de tout raconter.
-narrateur|La tartine.
-narrateur|La fraise.
-narrateur|La route.
 narrateur|Les mots montent très vite.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
-narrateur|Sarah tient le camion rouge.
-narrateur|Les roues sont encore froides.
-narrateur|Victorina ne dit rien.</t>
+enfant-f|Le rayon !
+enfant-f|Le tapis !
+enfant-f|Le camion !
+narrateur|Sarah pousse trop vite vers elle.
+narrateur|Le camion tape le sac.
+enfant-f|Oh.
+narrateur|Le camion bascule sur le parquet.
+enfant-f|Le camion.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Victorina, Sarah ?
+enfant-f|Oui, papa.
+maman|Tes mains tiennent le camion, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de parquet tremble, puis tient.
+narrateur|Victorina reste près du sac.
+enfant-f|Elle ne dit rien, papa.
+narrateur|Sarah regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>camion</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1428,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina parle peu. Que fait Sarah ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina parle peu. Que fait &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maya parle peu. Que fait Kenzo ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina parle peu. Que fait &lt;emphasis&gt;Sarah&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1466,7 +1496,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1477,7 +1507,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1492,34 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1534,17 +1568,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorina_parle_peu_que_fait_sarah; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1577,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah respire. Elle tend le camion. Pour toi. Elle attend. On n'entend plus que l'horloge. Victorina prend le camion. Elle ne dit rien. On ne force pas la parole. Regarder, c'est déjà jouer. Sarah pose encore un coussin. Victorina pousse le camion. Les roues font un petit bruit. La route grandit. Le garage se rapproche. Encore un coussin. Victorina le pose. Puis elle dit tout bas. Vroom. Vroom. Tu as su attendre. Bravo, Sarah. Le camion entre dans le garage. Toc. Il est arrivé. Sarah passe la main sur le toit. Le plastique est tiède.</t>
+          <t>Sarah veut le camion, tout de suite. Je le pousse, maintenant ! Elle avance trop vite vers Victorina. Les mots se bousculent dans sa bouche. Victorina baisse les yeux. Elle serre le sac contre elle. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le camion, un instant. Elle écoute le rayon sur le bois. Tu veux la route avec Victorina ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le camion, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle attend. Elle tend le camion. Pour toi. Victorina ne dit rien. Elle prend le camion, sans parler. Oui. Sarah pose les mains sur le tapis. Elle reste, sans se presser. Victorina pousse le camion, plus lentement. Merci, Sarah. Papa a vu les deux, au salon. Le poil est tiède, sous les doigts. Il est chaud. La route tient, un peu de travers. Le camion. Il a une porte, là ? Oui, là. Sarah glisse la main sur le toit. Le plastique est doux, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Victorina s'assoit, puis se relève. Vroom. On va jusqu'au bout ? Le tapis bleu va jusqu'au parquet. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah respire. Elle tend le camion. Pour toi. Elle attend. On n'entend plus que l'horloge. Victorina prend le camion. Elle ne dit rien. On ne force pas la parole. Regarder, c'est déjà jouer. Sarah pose encore un coussin. Victorina pousse le camion. Les roues font un petit bruit. La route grandit. Le garage se rapproche. Encore un coussin. Victorina le pose. Puis elle dit tout bas. Vroom. Vroom. Tu as su attendre. Bravo, Sarah. Le camion entre dans le garage. Toc. Il est arrivé. Sarah passe la main sur le toit. Le plastique est tiède.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut le &lt;emphasis level="moderate"&gt;camion&lt;/emphasis&gt;, tout de suite. Je le pousse, maintenant ! Elle avance trop vite vers Victorina. Les mots se bousculent dans sa bouche. Victorina baisse les yeux. Elle serre le sac contre elle. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le camion, un instant. Elle écoute le rayon sur le bois. Tu veux la route avec Victorina ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le camion, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle attend. Elle tend le camion. Pour toi. Victorina ne dit rien. Elle prend le camion, sans parler. Oui. Sarah pose les mains sur le tapis. Elle reste, sans se presser. Victorina pousse le camion, plus lentement. Merci, Sarah. Papa a vu les deux, au salon. Le poil est tiède, sous les doigts. Il est chaud. La route tient, un peu de travers. Le camion. Il a une porte, là ? Oui, là. Sarah glisse la main sur le toit. Le plastique est doux, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Victorina s'assoit, puis se relève. Vroom. On va jusqu'au bout ? Le tapis bleu va jusqu'au parquet. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kenzo a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Il a tendu un jouet. Maya a pris le camion. On n'a pas forcé la parole. [pause]</t>
+          <t>Sarah veut le &lt;emphasis&gt;camion&lt;/emphasis&gt;, tout de suite. Je le pousse, maintenant ! Elle avance trop vite vers Victorina. Les mots se bousculent dans sa bouche. Victorina baisse les yeux. Elle serre le sac contre elle. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le camion, un instant. Elle écoute le rayon sur le bois. Tu veux la route avec Victorina ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le camion, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle attend. Elle tend le camion. Pour toi. Victorina ne dit rien. Elle prend le camion, sans parler. Oui. Sarah pose les mains sur le tapis. Elle reste, sans se presser. Victorina pousse le camion, plus lentement. Merci, Sarah. Papa a vu les deux, au salon. Le poil est tiède, sous les doigts. Il est chaud. La route tient, un peu de travers. Le camion. Il a une porte, là ? Oui, là. Sarah glisse la main sur le toit. Le plastique est doux, contre la peau. Tes mains sont au chaud, Sarah ? Un peu, maman. Victorina s'assoit, puis se relève. Vroom. On va jusqu'au bout ? Le tapis bleu va jusqu'au parquet. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1702,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>camion</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1716,37 +1750,61 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_attend_tend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah respire.
+          <t>narrateur|Sarah veut le camion, tout de suite.
+enfant-f|Je le pousse, maintenant !
+narrateur|Elle avance trop vite vers Victorina.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Victorina baisse les yeux.
+narrateur|Elle serre le sac contre elle.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le camion, un instant.
+narrateur|Elle écoute le rayon sur le bois.
+papa|Tu veux la route avec Victorina ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose le camion, puis on reste.
+enfant-f|D'accord.
+narrateur|Sarah reste un moment, les mains ouvertes.
+narrateur|Elle attend.
 narrateur|Elle tend le camion.
 enfant-f|Pour toi.
-narrateur|Elle attend.
-narrateur|On n'entend plus que l'horloge.
-narrateur|Victorina prend le camion.
-narrateur|Elle ne dit rien.
-maman|On ne force pas la parole.
-papa|Regarder, c'est déjà jouer.
-narrateur|Sarah pose encore un coussin.
-narrateur|Victorina pousse le camion.
-narrateur|Les roues font un petit bruit.
-narrateur|La route grandit.
-narrateur|Le garage se rapproche.
-enfant-f|Encore un coussin.
-narrateur|Victorina le pose.
-narrateur|Puis elle dit tout bas.
-enfant-f|Vroom.
-enfant-f|Vroom.
-papa|Tu as su attendre.
-papa|Bravo, Sarah.
-narrateur|Le camion entre dans le garage.
-narrateur|Toc.
-maman|Il est arrivé.
-narrateur|Sarah passe la main sur le toit.
-narrateur|Le plastique est tiède.</t>
+narrateur|Victorina ne dit rien.
+narrateur|Elle prend le camion, sans parler.
+copine|Oui.
+narrateur|Sarah pose les mains sur le tapis.
+narrateur|Elle reste, sans se presser.
+narrateur|Victorina pousse le camion, plus lentement.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, au salon.
+maman|Le poil est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|La route tient, un peu de travers.
+enfant-f|Le camion.
+papa|Il a une porte, là ?
+enfant-f|Oui, là.
+narrateur|Sarah glisse la main sur le toit.
+narrateur|Le plastique est doux, contre la peau.
+maman|Tes mains sont au chaud, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Victorina s'assoit, puis se relève.
+copine|Vroom.
+enfant-f|On va jusqu'au bout ?
+maman|Le tapis bleu va jusqu'au parquet.
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tapis</t>
         </is>
       </c>
     </row>
@@ -1773,17 +1831,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman apporte deux tartines. La confiture brille encore. Vous voulez un goûter ? Victorina secoue la tête. D'accord. D'accord. Sarah croque un coin. Victorina reste près du garage. Elle tient encore le camion. Sarah attend. Puis Victorina s'assoit. Elle croque un morceau de pomme. Tu as fini ta route, Sarah ? Oui, maman. Le camion est au garage. Les miettes sont encore là. Le couvercle repose sur le pot. La fraise sent encore un peu.</t>
+          <t>Ils restent sur le tapis bleu. Une boîte en bois fait un garage. Il entre, maintenant ! Sarah pousse trop vite. Le camion penche vers le parquet. Ça tombe ! Victorina tend les mains, sans parler. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le camion, un instant. Elle écoute le silence du salon. Au bord du tapis, un éclat de parquet luit. Là, sur le bois. Tu prends le camion, Victorina ? Victorina ne dit rien. Elle tend les mains, sans parler. Oui. Sarah pousse le camion, sans se presser. Victorina le reçoit, plus lentement. Le plastique est lisse et tiède. Tu le vois, le camion ? Oui, papa. Le tapis bleu est près du parquet ? Oui, maman. Le camion entre dans la boîte. Sarah pose une main sur le toit. Victorina pose la suivante. La boîte tient, Sarah ? Oui, papa. Un rayon passe sur le parquet. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman apporte deux tartines. La confiture brille encore. Vous voulez un goûter ? Victorina secoue la tête. D'accord. D'accord. Sarah croque un coin. Victorina reste près du garage. Elle tient encore le camion. Sarah attend. Puis Victorina s'assoit. Elle croque un morceau de pomme. Tu as fini ta route, Sarah ? Oui, maman. Le camion est au garage. Les miettes sont encore là. Le couvercle repose sur le pot. La fraise sent encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent sur le tapis bleu. Une boîte en bois fait un garage. Il entre, maintenant ! Sarah pousse trop vite. Le camion penche vers le parquet. Ça tombe ! Victorina tend les mains, sans parler. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le camion, un instant. Elle écoute le silence du salon. Au bord du tapis, un &lt;emphasis level="moderate"&gt;éclat de parquet&lt;/emphasis&gt; luit. Là, sur le bois. Tu prends le camion, Victorina ? Victorina ne dit rien. Elle tend les mains, sans parler. Oui. Sarah pousse le camion, sans se presser. Victorina le reçoit, plus lentement. Le plastique est lisse et tiède. Tu le vois, le camion ? Oui, papa. Le tapis bleu est près du parquet ? Oui, maman. Le camion entre dans la boîte. Sarah pose une main sur le toit. Victorina pose la suivante. La boîte tient, Sarah ? Oui, papa. Un rayon passe sur le parquet. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Maya à mettre son manteau. Maya fait un petit signe de &lt;emphasis&gt;main&lt;/emphasis&gt;. Kenzo rend le camion. Il dit : à demain. [pause]</t>
+          <t>Ils restent sur le tapis bleu. Une boîte en bois fait un garage. Il entre, maintenant ! Sarah pousse trop vite. Le camion penche vers le parquet. Ça tombe ! Victorina tend les mains, sans parler. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le camion, un instant. Elle écoute le silence du salon. Au bord du tapis, un &lt;emphasis&gt;éclat de parquet&lt;/emphasis&gt; luit. Là, sur le bois. Tu prends le camion, Victorina ? Victorina ne dit rien. Elle tend les mains, sans parler. Oui. Sarah pousse le camion, sans se presser. Victorina le reçoit, plus lentement. Le plastique est lisse et tiède. Tu le vois, le camion ? Oui, papa. Le tapis bleu est près du parquet ? Oui, maman. Le camion entre dans la boîte. Sarah pose une main sur le toit. Victorina pose la suivante. La boîte tient, Sarah ? Oui, papa. Un rayon passe sur le parquet. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,7 +1888,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1838,10 +1896,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,30 +1922,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de parquet</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1954,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1910,27 +1968,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=boite_camion_trop_vite_elle_attend; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman apporte deux tartines.
-narrateur|La confiture brille encore.
-maman|Vous voulez un goûter ?
-narrateur|Victorina secoue la tête.
-enfant-f|D'accord.
-papa|D'accord.
-narrateur|Sarah croque un coin.
-narrateur|Victorina reste près du garage.
-narrateur|Elle tient encore le camion.
-narrateur|Sarah attend.
-narrateur|Puis Victorina s'assoit.
-narrateur|Elle croque un morceau de pomme.
-maman|Tu as fini ta route, Sarah ?
+          <t>narrateur|Ils restent sur le tapis bleu.
+narrateur|Une boîte en bois fait un garage.
+enfant-f|Il entre, maintenant !
+narrateur|Sarah pousse trop vite.
+narrateur|Le camion penche vers le parquet.
+enfant-f|Ça tombe !
+narrateur|Victorina tend les mains, sans parler.
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le camion, un instant.
+narrateur|Elle écoute le silence du salon.
+narrateur|Au bord du tapis, un éclat de parquet luit.
+enfant-f|Là, sur le bois.
+enfant-f|Tu prends le camion, Victorina ?
+narrateur|Victorina ne dit rien.
+narrateur|Elle tend les mains, sans parler.
+copine|Oui.
+narrateur|Sarah pousse le camion, sans se presser.
+narrateur|Victorina le reçoit, plus lentement.
+narrateur|Le plastique est lisse et tiède.
+papa|Tu le vois, le camion ?
+enfant-f|Oui, papa.
+maman|Le tapis bleu est près du parquet ?
 enfant-f|Oui, maman.
-enfant-f|Le camion est au garage.
-papa|Les miettes sont encore là.
-narrateur|Le couvercle repose sur le pot.
-narrateur|La fraise sent encore un peu.</t>
+narrateur|Le camion entre dans la boîte.
+narrateur|Sarah pose une main sur le toit.
+narrateur|Victorina pose la suivante.
+papa|La boîte tient, Sarah ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le parquet.
+enfant-f|Il allume le bois.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>boîte</t>
         </is>
       </c>
     </row>
@@ -1957,17 +2040,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le camion est arrivé. Au bout des coussins. La tartine est finie, aussi.</t>
+          <t>Ils restent près du tapis. Le camion est arrivé, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le plastique sent bon. Tu le sens, le camion ? Oui, maman. La route reste un peu, de travers. Elle a tenu, sur le tapis. Vroom. Le tapis est chaud, sous les mains. Le camion rouge fait de l'ombre. On y retourne, après. Un éclat de parquet tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le camion est arrivé. Au bout des coussins. La tartine est finie, aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du tapis. Le camion est arrivé, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le plastique sent bon. Tu le sens, le camion ? Oui, maman. La route reste un peu, de travers. Elle a tenu, sur le tapis. Vroom. Le tapis est chaud, sous les mains. Le camion rouge fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de parquet&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du tapis. Le camion est arrivé, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le plastique sent bon. Tu le sens, le camion ? Oui, maman. La route reste un peu, de travers. Elle a tenu, sur le tapis. Vroom. Le tapis est chaud, sous les mains. Le camion rouge fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de parquet&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2014,15 +2097,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2034,12 +2117,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2048,17 +2131,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de parquet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2067,11 +2154,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2080,26 +2167,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Le camion est arrivé.
-maman|Au bout des coussins.
-papa|La tartine est finie, aussi.</t>
+          <t>narrateur|Ils restent près du tapis.
+maman|Le camion est arrivé, Sarah ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Sarah souffle, un filet d'air.
+enfant-f|Le plastique sent bon.
+maman|Tu le sens, le camion ?
+enfant-f|Oui, maman.
+papa|La route reste un peu, de travers.
+enfant-f|Elle a tenu, sur le tapis.
+copine|Vroom.
+narrateur|Le tapis est chaud, sous les mains.
+narrateur|Le camion rouge fait de l'ombre.
+enfant-f|On y retourne, après.
+narrateur|Un éclat de parquet tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2177,6 +2281,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>